<commit_message>
memperbaiki font dan menampilkan produk agar sesuai resep bahan baku
</commit_message>
<xml_diff>
--- a/python/master_items_raw_updated.xlsx
+++ b/python/master_items_raw_updated.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\skripsi_forecasting\python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5BDA792-DADE-46B7-9424-B6B0D30B00E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94DDA81D-1D9B-44E1-880F-0C9C76551E3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="144">
   <si>
     <t>item_raw_id</t>
   </si>
@@ -147,9 +147,6 @@
   </si>
   <si>
     <t>Sunflower Oil</t>
-  </si>
-  <si>
-    <t>liter</t>
   </si>
   <si>
     <t>PT. Minyak Sehat Indonesia</t>
@@ -1395,10 +1392,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="D14" s="4">
         <v>300000</v>
@@ -1413,10 +1410,10 @@
         <v>3</v>
       </c>
       <c r="H14" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="I14" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>43</v>
       </c>
       <c r="J14" s="2" t="s">
         <v>15</v>
@@ -1428,10 +1425,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>44</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>45</v>
       </c>
       <c r="D15" s="7">
         <v>450</v>
@@ -1446,10 +1443,10 @@
         <v>31</v>
       </c>
       <c r="H15" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="I15" s="5" t="s">
         <v>46</v>
-      </c>
-      <c r="I15" s="5" t="s">
-        <v>47</v>
       </c>
       <c r="J15" s="5" t="s">
         <v>15</v>
@@ -1461,10 +1458,10 @@
         <v>15</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D16" s="4">
         <v>500</v>
@@ -1479,10 +1476,10 @@
         <v>25</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="J16" s="2" t="s">
         <v>15</v>
@@ -1494,10 +1491,10 @@
         <v>16</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D17" s="7">
         <v>550</v>
@@ -1512,10 +1509,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="J17" s="5" t="s">
         <v>15</v>
@@ -1527,10 +1524,10 @@
         <v>17</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D18" s="4">
         <v>700</v>
@@ -1545,10 +1542,10 @@
         <v>1</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J18" s="2" t="s">
         <v>15</v>
@@ -1560,10 +1557,10 @@
         <v>18</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D19" s="7">
         <v>900</v>
@@ -1578,10 +1575,10 @@
         <v>1</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I19" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="J19" s="5" t="s">
         <v>15</v>
@@ -1593,10 +1590,10 @@
         <v>19</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D20" s="4">
         <v>450</v>
@@ -1611,10 +1608,10 @@
         <v>6</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J20" s="2" t="s">
         <v>15</v>
@@ -1626,10 +1623,10 @@
         <v>20</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D21" s="7">
         <v>500</v>
@@ -1644,10 +1641,10 @@
         <v>7</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="J21" s="5" t="s">
         <v>15</v>
@@ -1659,10 +1656,10 @@
         <v>21</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D22" s="4">
         <v>550</v>
@@ -1677,7 +1674,7 @@
         <v>0</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>33</v>
@@ -1692,10 +1689,10 @@
         <v>22</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D23" s="7">
         <v>700</v>
@@ -1710,10 +1707,10 @@
         <v>1</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I23" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J23" s="5" t="s">
         <v>15</v>
@@ -1725,10 +1722,10 @@
         <v>23</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D24" s="4">
         <v>900</v>
@@ -1743,10 +1740,10 @@
         <v>1</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J24" s="2" t="s">
         <v>15</v>
@@ -1758,10 +1755,10 @@
         <v>24</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D25" s="7">
         <v>450</v>
@@ -1776,10 +1773,10 @@
         <v>5</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I25" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="J25" s="5" t="s">
         <v>15</v>
@@ -1791,10 +1788,10 @@
         <v>25</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D26" s="4">
         <v>500</v>
@@ -1809,10 +1806,10 @@
         <v>4</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J26" s="2" t="s">
         <v>15</v>
@@ -1824,10 +1821,10 @@
         <v>26</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D27" s="7">
         <v>550</v>
@@ -1842,10 +1839,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I27" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="J27" s="5" t="s">
         <v>15</v>
@@ -1857,10 +1854,10 @@
         <v>27</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D28" s="4">
         <v>700</v>
@@ -1875,10 +1872,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J28" s="2" t="s">
         <v>15</v>
@@ -1890,10 +1887,10 @@
         <v>28</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D29" s="7">
         <v>900</v>
@@ -1908,10 +1905,10 @@
         <v>1</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I29" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J29" s="5" t="s">
         <v>15</v>
@@ -1923,10 +1920,10 @@
         <v>29</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D30" s="4">
         <v>450</v>
@@ -1941,10 +1938,10 @@
         <v>4</v>
       </c>
       <c r="H30" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="I30" s="2" t="s">
         <v>76</v>
-      </c>
-      <c r="I30" s="2" t="s">
-        <v>77</v>
       </c>
       <c r="J30" s="2" t="s">
         <v>15</v>
@@ -1956,10 +1953,10 @@
         <v>30</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D31" s="7">
         <v>500</v>
@@ -1974,10 +1971,10 @@
         <v>4</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I31" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J31" s="5" t="s">
         <v>15</v>
@@ -1989,10 +1986,10 @@
         <v>31</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D32" s="4">
         <v>550</v>
@@ -2007,10 +2004,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J32" s="2" t="s">
         <v>15</v>
@@ -2022,10 +2019,10 @@
         <v>32</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D33" s="7">
         <v>700</v>
@@ -2040,10 +2037,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I33" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J33" s="5" t="s">
         <v>15</v>
@@ -2055,10 +2052,10 @@
         <v>33</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D34" s="4">
         <v>900</v>
@@ -2073,10 +2070,10 @@
         <v>1</v>
       </c>
       <c r="H34" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J34" s="2" t="s">
         <v>15</v>
@@ -2088,10 +2085,10 @@
         <v>34</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D35" s="7">
         <v>450</v>
@@ -2106,10 +2103,10 @@
         <v>5</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I35" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J35" s="5" t="s">
         <v>15</v>
@@ -2121,10 +2118,10 @@
         <v>35</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D36" s="4">
         <v>500</v>
@@ -2139,10 +2136,10 @@
         <v>3</v>
       </c>
       <c r="H36" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J36" s="2" t="s">
         <v>15</v>
@@ -2154,10 +2151,10 @@
         <v>36</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D37" s="7">
         <v>550</v>
@@ -2172,10 +2169,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I37" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J37" s="5" t="s">
         <v>15</v>
@@ -2187,10 +2184,10 @@
         <v>37</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D38" s="4">
         <v>700</v>
@@ -2205,10 +2202,10 @@
         <v>1</v>
       </c>
       <c r="H38" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="J38" s="2" t="s">
         <v>15</v>
@@ -2220,10 +2217,10 @@
         <v>38</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D39" s="7">
         <v>900</v>
@@ -2238,10 +2235,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I39" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="J39" s="5" t="s">
         <v>15</v>
@@ -2253,10 +2250,10 @@
         <v>39</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D40" s="7">
         <v>450</v>
@@ -2271,10 +2268,10 @@
         <v>4</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J40" s="2" t="s">
         <v>15</v>
@@ -2286,10 +2283,10 @@
         <v>40</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D41" s="4">
         <v>500</v>
@@ -2304,10 +2301,10 @@
         <v>2</v>
       </c>
       <c r="H41" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I41" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J41" s="5" t="s">
         <v>15</v>
@@ -2319,10 +2316,10 @@
         <v>41</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D42" s="7">
         <v>550</v>
@@ -2337,10 +2334,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J42" s="2" t="s">
         <v>15</v>
@@ -2352,10 +2349,10 @@
         <v>42</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D43" s="4">
         <v>700</v>
@@ -2370,10 +2367,10 @@
         <v>1</v>
       </c>
       <c r="H43" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I43" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="J43" s="5" t="s">
         <v>15</v>
@@ -2385,10 +2382,10 @@
         <v>43</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D44" s="7">
         <v>900</v>
@@ -2403,10 +2400,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="J44" s="2" t="s">
         <v>15</v>
@@ -2418,10 +2415,10 @@
         <v>44</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D45" s="7">
         <v>450</v>
@@ -2436,10 +2433,10 @@
         <v>2</v>
       </c>
       <c r="H45" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I45" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="J45" s="5" t="s">
         <v>15</v>
@@ -2451,10 +2448,10 @@
         <v>45</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D46" s="4">
         <v>500</v>
@@ -2469,10 +2466,10 @@
         <v>1</v>
       </c>
       <c r="H46" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="J46" s="2" t="s">
         <v>15</v>
@@ -2484,10 +2481,10 @@
         <v>46</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D47" s="7">
         <v>550</v>
@@ -2502,10 +2499,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I47" s="5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="J47" s="5" t="s">
         <v>15</v>
@@ -2517,10 +2514,10 @@
         <v>47</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D48" s="4">
         <v>700</v>
@@ -2535,10 +2532,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J48" s="2" t="s">
         <v>15</v>
@@ -2550,10 +2547,10 @@
         <v>48</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D49" s="7">
         <v>900</v>
@@ -2568,10 +2565,10 @@
         <v>1</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I49" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="J49" s="5" t="s">
         <v>15</v>
@@ -2583,10 +2580,10 @@
         <v>49</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D50" s="7">
         <v>450</v>
@@ -2601,10 +2598,10 @@
         <v>2</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I50" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="J50" s="5" t="s">
         <v>15</v>
@@ -2616,10 +2613,10 @@
         <v>50</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D51" s="4">
         <v>500</v>
@@ -2634,10 +2631,10 @@
         <v>1</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="J51" s="2" t="s">
         <v>15</v>
@@ -2649,10 +2646,10 @@
         <v>51</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D52" s="7">
         <v>550</v>
@@ -2667,10 +2664,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I52" s="5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="J52" s="5" t="s">
         <v>15</v>
@@ -2682,10 +2679,10 @@
         <v>52</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D53" s="4">
         <v>700</v>
@@ -2700,10 +2697,10 @@
         <v>1</v>
       </c>
       <c r="H53" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J53" s="2" t="s">
         <v>15</v>
@@ -2715,10 +2712,10 @@
         <v>53</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D54" s="7">
         <v>900</v>
@@ -2733,10 +2730,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I54" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="J54" s="5" t="s">
         <v>15</v>
@@ -2748,10 +2745,10 @@
         <v>54</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D55" s="7">
         <v>450</v>
@@ -2766,10 +2763,10 @@
         <v>2</v>
       </c>
       <c r="H55" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I55" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="J55" s="5" t="s">
         <v>15</v>
@@ -2781,10 +2778,10 @@
         <v>55</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D56" s="4">
         <v>500</v>
@@ -2799,10 +2796,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I56" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="J56" s="2" t="s">
         <v>15</v>
@@ -2814,10 +2811,10 @@
         <v>56</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D57" s="7">
         <v>550</v>
@@ -2832,10 +2829,10 @@
         <v>1</v>
       </c>
       <c r="H57" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I57" s="5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="J57" s="5" t="s">
         <v>15</v>
@@ -2847,10 +2844,10 @@
         <v>57</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D58" s="4">
         <v>700</v>
@@ -2865,10 +2862,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I58" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J58" s="2" t="s">
         <v>15</v>
@@ -2880,10 +2877,10 @@
         <v>58</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D59" s="7">
         <v>900</v>
@@ -2898,10 +2895,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I59" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="J59" s="5" t="s">
         <v>15</v>
@@ -2913,7 +2910,7 @@
         <v>59</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C60" s="2" t="s">
         <v>12</v>
@@ -2934,7 +2931,7 @@
         <v>13</v>
       </c>
       <c r="I60" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J60" s="2" t="s">
         <v>15</v>
@@ -2946,7 +2943,7 @@
         <v>60</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C61" s="5" t="s">
         <v>12</v>
@@ -2967,7 +2964,7 @@
         <v>13</v>
       </c>
       <c r="I61" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J61" s="5" t="s">
         <v>15</v>
@@ -2979,7 +2976,7 @@
         <v>61</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C62" s="2" t="s">
         <v>12</v>
@@ -3000,7 +2997,7 @@
         <v>13</v>
       </c>
       <c r="I62" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="J62" s="2" t="s">
         <v>15</v>
@@ -3012,7 +3009,7 @@
         <v>62</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C63" s="5" t="s">
         <v>12</v>
@@ -3033,7 +3030,7 @@
         <v>13</v>
       </c>
       <c r="I63" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J63" s="5" t="s">
         <v>15</v>
@@ -3045,7 +3042,7 @@
         <v>63</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C64" s="2" t="s">
         <v>12</v>
@@ -3066,7 +3063,7 @@
         <v>13</v>
       </c>
       <c r="I64" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="J64" s="2" t="s">
         <v>15</v>
@@ -3100,7 +3097,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="18.5" x14ac:dyDescent="0.35">
       <c r="A1" s="18" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B1" s="16"/>
       <c r="C1" s="16"/>
@@ -3112,7 +3109,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="17" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B2" s="16"/>
       <c r="C2" s="16"/>
@@ -3124,7 +3121,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B3" s="16"/>
       <c r="C3" s="16"/>
@@ -3136,28 +3133,28 @@
     </row>
     <row r="5" spans="1:8" ht="35" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="B5" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="C5" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="D5" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="E5" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="F5" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="G5" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="H5" s="8" t="s">
         <v>142</v>
-      </c>
-      <c r="H5" s="8" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
@@ -3503,7 +3500,7 @@
         <v>14</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C19" s="14">
         <v>4.3973000000000004</v>
@@ -3529,7 +3526,7 @@
         <v>15</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C20" s="11">
         <v>4.4794999999999998</v>
@@ -3555,7 +3552,7 @@
         <v>16</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C21" s="14">
         <v>0</v>
@@ -3581,7 +3578,7 @@
         <v>17</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C22" s="11">
         <v>1.6400000000000001E-2</v>
@@ -3607,7 +3604,7 @@
         <v>18</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C23" s="14">
         <v>2.7000000000000001E-3</v>
@@ -3633,7 +3630,7 @@
         <v>19</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C24" s="11">
         <v>0.8</v>
@@ -3659,7 +3656,7 @@
         <v>20</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C25" s="14">
         <v>0.67669999999999997</v>
@@ -3685,7 +3682,7 @@
         <v>21</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C26" s="11">
         <v>0</v>
@@ -3711,7 +3708,7 @@
         <v>22</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C27" s="14">
         <v>1.37E-2</v>
@@ -3737,7 +3734,7 @@
         <v>23</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C28" s="11">
         <v>8.2000000000000007E-3</v>
@@ -3763,7 +3760,7 @@
         <v>24</v>
       </c>
       <c r="B29" s="13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C29" s="14">
         <v>0.40550000000000003</v>
@@ -3789,7 +3786,7 @@
         <v>25</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C30" s="11">
         <v>0.3014</v>
@@ -3815,7 +3812,7 @@
         <v>26</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C31" s="14">
         <v>0</v>
@@ -3841,7 +3838,7 @@
         <v>27</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C32" s="11">
         <v>0</v>
@@ -3867,7 +3864,7 @@
         <v>28</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C33" s="14">
         <v>2.7000000000000001E-3</v>
@@ -3893,7 +3890,7 @@
         <v>29</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C34" s="11">
         <v>0.46300000000000002</v>
@@ -3919,7 +3916,7 @@
         <v>30</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C35" s="14">
         <v>0.34520000000000001</v>
@@ -3945,7 +3942,7 @@
         <v>31</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C36" s="11">
         <v>0</v>
@@ -3971,7 +3968,7 @@
         <v>32</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C37" s="14">
         <v>0</v>
@@ -3997,7 +3994,7 @@
         <v>33</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C38" s="11">
         <v>2.7000000000000001E-3</v>
@@ -4023,7 +4020,7 @@
         <v>34</v>
       </c>
       <c r="B39" s="13" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C39" s="14">
         <v>0.41099999999999998</v>
@@ -4049,7 +4046,7 @@
         <v>35</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C40" s="11">
         <v>0.28220000000000001</v>
@@ -4075,7 +4072,7 @@
         <v>36</v>
       </c>
       <c r="B41" s="13" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C41" s="14">
         <v>0</v>
@@ -4101,7 +4098,7 @@
         <v>37</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C42" s="11">
         <v>5.4999999999999997E-3</v>
@@ -4127,7 +4124,7 @@
         <v>38</v>
       </c>
       <c r="B43" s="13" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C43" s="14">
         <v>0</v>
@@ -4153,7 +4150,7 @@
         <v>39</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C44" s="11">
         <v>0.43009999999999998</v>
@@ -4179,7 +4176,7 @@
         <v>40</v>
       </c>
       <c r="B45" s="13" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C45" s="14">
         <v>0.21099999999999999</v>
@@ -4205,7 +4202,7 @@
         <v>41</v>
       </c>
       <c r="B46" s="10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C46" s="11">
         <v>0</v>
@@ -4231,7 +4228,7 @@
         <v>42</v>
       </c>
       <c r="B47" s="13" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C47" s="14">
         <v>5.4999999999999997E-3</v>
@@ -4257,7 +4254,7 @@
         <v>43</v>
       </c>
       <c r="B48" s="10" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C48" s="11">
         <v>0</v>
@@ -4283,7 +4280,7 @@
         <v>44</v>
       </c>
       <c r="B49" s="13" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C49" s="14">
         <v>9.8599999999999993E-2</v>
@@ -4309,7 +4306,7 @@
         <v>45</v>
       </c>
       <c r="B50" s="10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C50" s="11">
         <v>4.9299999999999997E-2</v>
@@ -4335,7 +4332,7 @@
         <v>46</v>
       </c>
       <c r="B51" s="13" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C51" s="14">
         <v>0</v>
@@ -4361,7 +4358,7 @@
         <v>47</v>
       </c>
       <c r="B52" s="10" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C52" s="11">
         <v>0</v>
@@ -4387,7 +4384,7 @@
         <v>48</v>
       </c>
       <c r="B53" s="13" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C53" s="14">
         <v>2.7000000000000001E-3</v>
@@ -4413,7 +4410,7 @@
         <v>49</v>
       </c>
       <c r="B54" s="10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C54" s="11">
         <v>8.2199999999999995E-2</v>
@@ -4439,7 +4436,7 @@
         <v>50</v>
       </c>
       <c r="B55" s="13" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C55" s="14">
         <v>3.2899999999999999E-2</v>
@@ -4465,7 +4462,7 @@
         <v>51</v>
       </c>
       <c r="B56" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C56" s="11">
         <v>0</v>
@@ -4491,7 +4488,7 @@
         <v>52</v>
       </c>
       <c r="B57" s="13" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C57" s="14">
         <v>2.7000000000000001E-3</v>
@@ -4517,7 +4514,7 @@
         <v>53</v>
       </c>
       <c r="B58" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C58" s="11">
         <v>0</v>
@@ -4543,7 +4540,7 @@
         <v>54</v>
       </c>
       <c r="B59" s="13" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C59" s="14">
         <v>0.126</v>
@@ -4569,7 +4566,7 @@
         <v>55</v>
       </c>
       <c r="B60" s="10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C60" s="11">
         <v>0</v>
@@ -4595,7 +4592,7 @@
         <v>56</v>
       </c>
       <c r="B61" s="13" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C61" s="14">
         <v>6.3E-2</v>
@@ -4621,7 +4618,7 @@
         <v>57</v>
       </c>
       <c r="B62" s="10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C62" s="11">
         <v>0</v>
@@ -4647,7 +4644,7 @@
         <v>58</v>
       </c>
       <c r="B63" s="13" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C63" s="14">
         <v>0</v>
@@ -4673,7 +4670,7 @@
         <v>59</v>
       </c>
       <c r="B64" s="10" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C64" s="11">
         <v>7.2521000000000004</v>
@@ -4699,7 +4696,7 @@
         <v>60</v>
       </c>
       <c r="B65" s="13" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C65" s="14">
         <v>6.8521000000000001</v>
@@ -4725,7 +4722,7 @@
         <v>61</v>
       </c>
       <c r="B66" s="10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C66" s="11">
         <v>6.3E-2</v>
@@ -4751,7 +4748,7 @@
         <v>62</v>
       </c>
       <c r="B67" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C67" s="14">
         <v>4.3799999999999999E-2</v>
@@ -4777,7 +4774,7 @@
         <v>63</v>
       </c>
       <c r="B68" s="10" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C68" s="11">
         <v>1.9199999999999998E-2</v>

</xml_diff>